<commit_message>
Convert manuscript to Quarto (ms.qmd) with BibTeX references
Converted ms-2026-09-13v2.docx to ms.qmd. Citations use keys from ref.bib
(exported from Zotero, plus DeWeerd 2022 and Lawson 2020 added by hand).
Figures are cross-referenced Quarto figure divs. Table 1 is read from
table_1_autogenerated_edited.xlsx at render time. Word comments are kept
as callout-note blocks. Rendered ms.pdf and ms.docx included.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EFy9SMD2JCfkeBQtpG3xaT
</commit_message>
<xml_diff>
--- a/table_1_autogenerated_edited.xlsx
+++ b/table_1_autogenerated_edited.xlsx
@@ -22,25 +22,26 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="124">
   <si>
-    <t xml:space="preserve">89-Type Classification Signature ID</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cosine vs Extracted 476-Type Sig Collapsed to 89-Type</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cosine 89-Type Sig vs BestMatch89 Spectrum</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Closest Koh et al. Sig</t>
+    <t xml:space="preserve">89-Type
+Signature ID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cosine 476-Type Sig Collapsed to 89-Type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cosine 89-Type Sig vs Best Match Spectrum</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Koh et al. Sig</t>
   </si>
   <si>
     <t xml:space="preserve">Cosine 89-Type Sig vs Koh et al.</t>
   </si>
   <si>
-    <t xml:space="preserve">Extracted 83-Type Sig ID</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Closest Jin et al. Sig</t>
+    <t xml:space="preserve">83-Type Sig ID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jin et al. Sig</t>
   </si>
   <si>
     <t xml:space="preserve">Cosine vs Jin et al.</t>
@@ -442,9 +443,9 @@
     </font>
     <font>
       <b val="true"/>
-      <sz val="8"/>
+      <sz val="11"/>
       <color rgb="FF000000"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
     </font>
@@ -464,12 +465,21 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="hair"/>
+      <right style="hair"/>
+      <top style="hair"/>
+      <bottom style="hair">
+        <color rgb="FF666666"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -498,60 +508,64 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -612,7 +626,7 @@
       <rgbColor rgb="FFFFCC00"/>
       <rgbColor rgb="FFFF9900"/>
       <rgbColor rgb="FFFF6600"/>
-      <rgbColor rgb="FF666699"/>
+      <rgbColor rgb="FF666666"/>
       <rgbColor rgb="FF969696"/>
       <rgbColor rgb="FF003366"/>
       <rgbColor rgb="FF339966"/>
@@ -810,993 +824,994 @@
   <dimension ref="A1:H45"/>
   <sheetFormatPr defaultColWidth="11.0546875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="2" min="1" style="1" width="11.05"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="9.11"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11.05"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="11.05"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="2" width="9.11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="6.61"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="8.45"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="7.58"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="7.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="6.83"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="5.2"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="18" min="9" style="2" width="11.05"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="2" width="5.2"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="18" min="9" style="3" width="11.05"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16374" min="19" style="1" width="11.05"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16375" style="1" width="11.53"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="46.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="3" t="s">
+    <row r="1" customFormat="false" ht="67.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="H1" s="5" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="5" t="n">
+      <c r="B2" s="7" t="n">
         <v>0.992255142965221</v>
       </c>
-      <c r="C2" s="5" t="n">
+      <c r="C2" s="7" t="n">
         <v>0.983074166206997</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="E2" s="7" t="n">
+      <c r="E2" s="9" t="n">
         <v>0.902299690593055</v>
       </c>
-      <c r="F2" s="8" t="s">
+      <c r="F2" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="G2" s="8" t="s">
+      <c r="G2" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="H2" s="9" t="n">
+      <c r="H2" s="11" t="n">
         <v>0.984922448681081</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="5" t="n">
+      <c r="B3" s="7" t="n">
         <v>0.992510044644143</v>
       </c>
-      <c r="C3" s="5" t="n">
+      <c r="C3" s="7" t="n">
         <v>0.984963987993242</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="D3" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="E3" s="5" t="n">
+      <c r="E3" s="7" t="n">
         <v>0.979574035881082</v>
       </c>
-      <c r="F3" s="8" t="s">
+      <c r="F3" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="G3" s="8" t="s">
+      <c r="G3" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="H3" s="9" t="n">
+      <c r="H3" s="11" t="n">
         <v>0.984922448681081</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="B4" s="5" t="n">
+      <c r="B4" s="7" t="n">
         <v>0.981866375036531</v>
       </c>
-      <c r="C4" s="5" t="n">
+      <c r="C4" s="7" t="n">
         <v>0.967513714201868</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="E4" s="5" t="n">
+      <c r="E4" s="7" t="n">
         <v>0.941518994814764</v>
       </c>
-      <c r="F4" s="8" t="s">
+      <c r="F4" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="G4" s="8" t="s">
+      <c r="G4" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="H4" s="9" t="n">
+      <c r="H4" s="11" t="n">
         <v>0.984922448681081</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="B5" s="5" t="n">
+      <c r="B5" s="7" t="n">
         <v>0.985294551259857</v>
       </c>
-      <c r="C5" s="5" t="n">
+      <c r="C5" s="7" t="n">
         <v>0.971029412189185</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="D5" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="E5" s="5" t="n">
+      <c r="E5" s="7" t="n">
         <v>0.982386172138281</v>
       </c>
-      <c r="F5" s="8" t="s">
+      <c r="F5" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="G5" s="8" t="s">
+      <c r="G5" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="H5" s="9" t="n">
+      <c r="H5" s="11" t="n">
         <v>0.993151664747609</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="B6" s="5" t="n">
+      <c r="B6" s="7" t="n">
         <v>0.985774870351135</v>
       </c>
-      <c r="C6" s="5" t="n">
+      <c r="C6" s="7" t="n">
         <v>0.964494916609992</v>
       </c>
-      <c r="D6" s="4"/>
-      <c r="E6" s="5"/>
-      <c r="F6" s="8" t="s">
+      <c r="D6" s="6"/>
+      <c r="E6" s="7"/>
+      <c r="F6" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="G6" s="8" t="s">
+      <c r="G6" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="H6" s="9" t="n">
+      <c r="H6" s="11" t="n">
         <v>0.993151664747609</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="B7" s="5" t="n">
+      <c r="B7" s="7" t="n">
         <v>0.984219621422622</v>
       </c>
-      <c r="C7" s="5" t="n">
+      <c r="C7" s="7" t="n">
         <v>0.974439597175431</v>
       </c>
-      <c r="D7" s="4"/>
-      <c r="E7" s="5"/>
-      <c r="F7" s="8" t="s">
+      <c r="D7" s="6"/>
+      <c r="E7" s="7"/>
+      <c r="F7" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="G7" s="8" t="s">
+      <c r="G7" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="H7" s="9" t="n">
+      <c r="H7" s="11" t="n">
         <v>0.993151664747609</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4" t="s">
+      <c r="A8" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="B8" s="5" t="n">
+      <c r="B8" s="7" t="n">
         <v>0.951485193101285</v>
       </c>
-      <c r="C8" s="5" t="n">
+      <c r="C8" s="7" t="n">
         <v>0.973836073710126</v>
       </c>
-      <c r="D8" s="4"/>
-      <c r="E8" s="5"/>
-      <c r="F8" s="8" t="s">
+      <c r="D8" s="6"/>
+      <c r="E8" s="7"/>
+      <c r="F8" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="G8" s="8" t="s">
+      <c r="G8" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="H8" s="9" t="n">
+      <c r="H8" s="11" t="n">
         <v>0.940287785333133</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4" t="s">
+      <c r="A9" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="B9" s="5" t="n">
+      <c r="B9" s="7" t="n">
         <v>0.996989105749797</v>
       </c>
-      <c r="C9" s="5" t="n">
+      <c r="C9" s="7" t="n">
         <v>0.995211832210858</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="D9" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="E9" s="5" t="n">
+      <c r="E9" s="7" t="n">
         <v>0.952660131921794</v>
       </c>
-      <c r="F9" s="8" t="s">
+      <c r="F9" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="G9" s="8" t="s">
+      <c r="G9" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="H9" s="9" t="n">
+      <c r="H9" s="11" t="n">
         <v>0.940287785333133</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4" t="s">
+      <c r="A10" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="B10" s="5" t="n">
+      <c r="B10" s="7" t="n">
         <v>0.995469500627484</v>
       </c>
-      <c r="C10" s="5" t="n">
+      <c r="C10" s="7" t="n">
         <v>0.984487609190074</v>
       </c>
-      <c r="D10" s="4" t="s">
+      <c r="D10" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="E10" s="5" t="n">
+      <c r="E10" s="7" t="n">
         <v>0.982035840349706</v>
       </c>
-      <c r="F10" s="4" t="s">
+      <c r="F10" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="G10" s="4"/>
-      <c r="H10" s="5"/>
+      <c r="G10" s="6"/>
+      <c r="H10" s="7"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="s">
+      <c r="A11" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="B11" s="10" t="n">
+      <c r="B11" s="7" t="n">
         <v>0.998300405557043</v>
       </c>
-      <c r="C11" s="10" t="n">
+      <c r="C11" s="7" t="n">
         <v>0.990772393970387</v>
       </c>
-      <c r="D11" s="4" t="s">
+      <c r="D11" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="E11" s="11"/>
-      <c r="F11" s="8" t="s">
+      <c r="E11" s="12"/>
+      <c r="F11" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="G11" s="8"/>
-      <c r="H11" s="12"/>
+      <c r="G11" s="10"/>
+      <c r="H11" s="11"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="4" t="s">
+      <c r="A12" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="B12" s="10" t="n">
+      <c r="B12" s="7" t="n">
         <v>0.995334578633942</v>
       </c>
-      <c r="C12" s="10" t="n">
+      <c r="C12" s="7" t="n">
         <v>0.982577764655484</v>
       </c>
-      <c r="D12" s="4"/>
-      <c r="E12" s="11"/>
-      <c r="F12" s="8" t="s">
+      <c r="D12" s="6"/>
+      <c r="E12" s="12"/>
+      <c r="F12" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="G12" s="8"/>
-      <c r="H12" s="12"/>
+      <c r="G12" s="10"/>
+      <c r="H12" s="11"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="4" t="s">
+      <c r="A13" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="B13" s="10" t="n">
+      <c r="B13" s="7" t="n">
         <v>0.957464770264216</v>
       </c>
-      <c r="C13" s="10" t="n">
+      <c r="C13" s="7" t="n">
         <v>0.93439271726825</v>
       </c>
-      <c r="D13" s="4"/>
-      <c r="E13" s="10"/>
-      <c r="F13" s="8" t="s">
+      <c r="D13" s="6"/>
+      <c r="E13" s="13"/>
+      <c r="F13" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="G13" s="8"/>
-      <c r="H13" s="12"/>
+      <c r="G13" s="10"/>
+      <c r="H13" s="11"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="4" t="s">
+      <c r="A14" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="B14" s="10" t="n">
+      <c r="B14" s="7" t="n">
         <v>0.998146875730815</v>
       </c>
-      <c r="C14" s="10" t="n">
+      <c r="C14" s="7" t="n">
         <v>0.994938158413937</v>
       </c>
-      <c r="D14" s="4" t="s">
+      <c r="D14" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="E14" s="10" t="n">
+      <c r="E14" s="13" t="n">
         <v>0.974493621233503</v>
       </c>
-      <c r="F14" s="4" t="s">
+      <c r="F14" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="G14" s="4" t="s">
+      <c r="G14" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="H14" s="10" t="n">
+      <c r="H14" s="7" t="n">
         <v>0.915585975794971</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="4" t="s">
+      <c r="A15" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="B15" s="10" t="n">
+      <c r="B15" s="7" t="n">
         <v>0.997720158832099</v>
       </c>
-      <c r="C15" s="10" t="n">
+      <c r="C15" s="7" t="n">
         <v>0.996684575925649</v>
       </c>
-      <c r="D15" s="4" t="s">
+      <c r="D15" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="E15" s="10" t="n">
+      <c r="E15" s="13" t="n">
         <v>0.979743627798565</v>
       </c>
-      <c r="F15" s="4" t="s">
+      <c r="F15" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="G15" s="4"/>
-      <c r="H15" s="10"/>
+      <c r="G15" s="6"/>
+      <c r="H15" s="7"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="4" t="s">
+      <c r="A16" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="B16" s="10" t="n">
+      <c r="B16" s="7" t="n">
         <v>0.994244385580007</v>
       </c>
-      <c r="C16" s="10" t="n">
+      <c r="C16" s="7" t="n">
         <v>0.991418420322135</v>
       </c>
-      <c r="D16" s="4" t="s">
+      <c r="D16" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E16" s="10" t="n">
+      <c r="E16" s="13" t="n">
         <v>0.981178677269259</v>
       </c>
-      <c r="F16" s="4" t="s">
+      <c r="F16" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="G16" s="4" t="s">
+      <c r="G16" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="H16" s="10" t="n">
+      <c r="H16" s="7" t="n">
         <v>0.968325983966513</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="4" t="s">
+      <c r="A17" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="B17" s="10" t="n">
+      <c r="B17" s="7" t="n">
         <v>0.999233941698574</v>
       </c>
-      <c r="C17" s="10" t="n">
+      <c r="C17" s="7" t="n">
         <v>0.925869317999378</v>
       </c>
-      <c r="D17" s="4" t="s">
+      <c r="D17" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="E17" s="10" t="n">
+      <c r="E17" s="13" t="n">
         <v>0.916987691367188</v>
       </c>
-      <c r="F17" s="4" t="s">
+      <c r="F17" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="G17" s="4"/>
-      <c r="H17" s="10"/>
+      <c r="G17" s="6"/>
+      <c r="H17" s="7"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="4" t="s">
+      <c r="A18" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="B18" s="10" t="n">
+      <c r="B18" s="7" t="n">
         <v>0.956900113069297</v>
       </c>
-      <c r="C18" s="10" t="n">
+      <c r="C18" s="7" t="n">
         <v>0.845720421013182</v>
       </c>
-      <c r="D18" s="4"/>
-      <c r="E18" s="10"/>
-      <c r="F18" s="4" t="s">
+      <c r="D18" s="6"/>
+      <c r="E18" s="13"/>
+      <c r="F18" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="G18" s="4" t="s">
+      <c r="G18" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="H18" s="10" t="n">
+      <c r="H18" s="7" t="n">
         <v>0.901574093270865</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="4" t="s">
+      <c r="A19" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="B19" s="10" t="n">
+      <c r="B19" s="7" t="n">
         <v>0.999980561669705</v>
       </c>
-      <c r="C19" s="10" t="n">
+      <c r="C19" s="7" t="n">
         <v>0.999995230749492</v>
       </c>
-      <c r="D19" s="4"/>
-      <c r="E19" s="10"/>
-      <c r="F19" s="4" t="s">
+      <c r="D19" s="6"/>
+      <c r="E19" s="13"/>
+      <c r="F19" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="G19" s="4" t="s">
+      <c r="G19" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="H19" s="10" t="n">
+      <c r="H19" s="7" t="n">
         <v>0.997513023161577</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="4" t="s">
+      <c r="A20" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="B20" s="10" t="n">
+      <c r="B20" s="7" t="n">
         <v>0.990839010473006</v>
       </c>
-      <c r="C20" s="10" t="n">
+      <c r="C20" s="7" t="n">
         <v>0.970118693726864</v>
       </c>
-      <c r="D20" s="4"/>
-      <c r="E20" s="10"/>
-      <c r="F20" s="4" t="s">
+      <c r="D20" s="6"/>
+      <c r="E20" s="13"/>
+      <c r="F20" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="G20" s="4" t="s">
+      <c r="G20" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="H20" s="10" t="n">
+      <c r="H20" s="7" t="n">
         <v>0.936826633707368</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="4" t="s">
+      <c r="A21" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="B21" s="10" t="n">
+      <c r="B21" s="7" t="n">
         <v>0.996183376620369</v>
       </c>
-      <c r="C21" s="10" t="n">
+      <c r="C21" s="7" t="n">
         <v>0.990794528992823</v>
       </c>
-      <c r="D21" s="4" t="s">
+      <c r="D21" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="E21" s="10" t="n">
+      <c r="E21" s="13" t="n">
         <v>0.988609053466361</v>
       </c>
-      <c r="F21" s="4" t="s">
+      <c r="F21" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="G21" s="4" t="s">
+      <c r="G21" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="H21" s="10" t="n">
+      <c r="H21" s="7" t="n">
         <v>0.958027842855097</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="4" t="s">
+      <c r="A22" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="B22" s="10" t="n">
+      <c r="B22" s="7" t="n">
         <v>0.988147727632474</v>
       </c>
-      <c r="C22" s="10" t="n">
+      <c r="C22" s="7" t="n">
         <v>0.994521225326853</v>
       </c>
-      <c r="D22" s="4" t="s">
+      <c r="D22" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="E22" s="10" t="n">
+      <c r="E22" s="13" t="n">
         <v>0.983091970341539</v>
       </c>
-      <c r="F22" s="4" t="s">
+      <c r="F22" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="G22" s="4" t="s">
+      <c r="G22" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="H22" s="10" t="n">
+      <c r="H22" s="7" t="n">
         <v>0.95838127103415</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="4" t="s">
+      <c r="A23" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="B23" s="10" t="n">
+      <c r="B23" s="7" t="n">
         <v>0.999977796576728</v>
       </c>
-      <c r="C23" s="10" t="n">
+      <c r="C23" s="7" t="n">
         <v>0.997152554293266</v>
       </c>
-      <c r="D23" s="4"/>
-      <c r="E23" s="10"/>
-      <c r="F23" s="4" t="s">
+      <c r="D23" s="6"/>
+      <c r="E23" s="13"/>
+      <c r="F23" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="G23" s="4"/>
-      <c r="H23" s="10"/>
+      <c r="G23" s="6"/>
+      <c r="H23" s="7"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="4" t="s">
+      <c r="A24" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="B24" s="10" t="n">
+      <c r="B24" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="C24" s="10" t="n">
+      <c r="C24" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="D24" s="4"/>
-      <c r="E24" s="10"/>
-      <c r="F24" s="4" t="s">
+      <c r="D24" s="6"/>
+      <c r="E24" s="13"/>
+      <c r="F24" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="G24" s="4"/>
-      <c r="H24" s="10"/>
+      <c r="G24" s="6"/>
+      <c r="H24" s="7"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="4" t="s">
+      <c r="A25" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="B25" s="10" t="n">
+      <c r="B25" s="7" t="n">
         <v>0.999970153131709</v>
       </c>
-      <c r="C25" s="10" t="n">
+      <c r="C25" s="7" t="n">
         <v>0.999914468410852</v>
       </c>
-      <c r="D25" s="4"/>
-      <c r="E25" s="10"/>
-      <c r="F25" s="4" t="s">
+      <c r="D25" s="6"/>
+      <c r="E25" s="13"/>
+      <c r="F25" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="G25" s="4"/>
-      <c r="H25" s="10"/>
+      <c r="G25" s="6"/>
+      <c r="H25" s="7"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="4" t="s">
+      <c r="A26" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="B26" s="10" t="n">
+      <c r="B26" s="7" t="n">
         <v>0.999368075167037</v>
       </c>
-      <c r="C26" s="10" t="n">
+      <c r="C26" s="7" t="n">
         <v>0.995835062831407</v>
       </c>
-      <c r="D26" s="4" t="s">
+      <c r="D26" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="E26" s="10" t="n">
+      <c r="E26" s="13" t="n">
         <v>0.995865147469362</v>
       </c>
-      <c r="F26" s="4" t="s">
+      <c r="F26" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="G26" s="4" t="s">
+      <c r="G26" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="H26" s="10" t="n">
+      <c r="H26" s="7" t="n">
         <v>0.908745879538509</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="4" t="s">
+      <c r="A27" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="B27" s="10" t="n">
+      <c r="B27" s="7" t="n">
         <v>0.991323935580266</v>
       </c>
-      <c r="C27" s="10" t="n">
+      <c r="C27" s="7" t="n">
         <v>0.949421224357304</v>
       </c>
-      <c r="D27" s="4"/>
-      <c r="E27" s="10"/>
-      <c r="F27" s="8" t="s">
+      <c r="D27" s="6"/>
+      <c r="E27" s="13"/>
+      <c r="F27" s="10" t="s">
         <v>80</v>
       </c>
-      <c r="G27" s="8"/>
-      <c r="H27" s="12"/>
+      <c r="G27" s="10"/>
+      <c r="H27" s="11"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="4" t="s">
+      <c r="A28" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="B28" s="10" t="n">
+      <c r="B28" s="7" t="n">
         <v>0.994265742578395</v>
       </c>
-      <c r="C28" s="10" t="n">
+      <c r="C28" s="7" t="n">
         <v>0.99220397390673</v>
       </c>
-      <c r="D28" s="4"/>
-      <c r="E28" s="10"/>
-      <c r="F28" s="8" t="s">
+      <c r="D28" s="6"/>
+      <c r="E28" s="13"/>
+      <c r="F28" s="10" t="s">
         <v>80</v>
       </c>
-      <c r="G28" s="8"/>
-      <c r="H28" s="12"/>
+      <c r="G28" s="10"/>
+      <c r="H28" s="11"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="4" t="s">
+      <c r="A29" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="B29" s="10" t="n">
+      <c r="B29" s="7" t="n">
         <v>0.994537961750642</v>
       </c>
-      <c r="C29" s="10" t="n">
+      <c r="C29" s="7" t="n">
         <v>0.96057484601985</v>
       </c>
-      <c r="D29" s="4"/>
-      <c r="E29" s="10"/>
-      <c r="F29" s="4" t="s">
+      <c r="D29" s="6"/>
+      <c r="E29" s="13"/>
+      <c r="F29" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="G29" s="4"/>
-      <c r="H29" s="10"/>
+      <c r="G29" s="6"/>
+      <c r="H29" s="7"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="4" t="s">
+      <c r="A30" s="6" t="s">
         <v>84</v>
       </c>
-      <c r="B30" s="10" t="n">
+      <c r="B30" s="7" t="n">
         <v>0.997211203480939</v>
       </c>
-      <c r="C30" s="10" t="n">
+      <c r="C30" s="7" t="n">
         <v>0.809677297640414</v>
       </c>
-      <c r="D30" s="4"/>
-      <c r="E30" s="10"/>
-      <c r="F30" s="8" t="s">
+      <c r="D30" s="6"/>
+      <c r="E30" s="13"/>
+      <c r="F30" s="10" t="s">
         <v>85</v>
       </c>
-      <c r="G30" s="8"/>
-      <c r="H30" s="12"/>
+      <c r="G30" s="10"/>
+      <c r="H30" s="11"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="4" t="s">
+      <c r="A31" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="B31" s="10" t="n">
+      <c r="B31" s="7" t="n">
         <v>0.979201595130134</v>
       </c>
-      <c r="C31" s="10" t="n">
+      <c r="C31" s="7" t="n">
         <v>0.936066840683912</v>
       </c>
-      <c r="D31" s="4" t="s">
+      <c r="D31" s="6" t="s">
         <v>87</v>
       </c>
-      <c r="E31" s="10" t="n">
+      <c r="E31" s="13" t="n">
         <v>0.965031393233845</v>
       </c>
-      <c r="F31" s="8" t="s">
+      <c r="F31" s="10" t="s">
         <v>85</v>
       </c>
-      <c r="G31" s="8"/>
-      <c r="H31" s="12"/>
+      <c r="G31" s="10"/>
+      <c r="H31" s="11"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="4" t="s">
+      <c r="A32" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="B32" s="10" t="n">
+      <c r="B32" s="7" t="n">
         <v>0.99194648722922</v>
       </c>
-      <c r="C32" s="10" t="n">
+      <c r="C32" s="7" t="n">
         <v>0.987166551716017</v>
       </c>
-      <c r="D32" s="4"/>
-      <c r="E32" s="10"/>
-      <c r="F32" s="4" t="s">
+      <c r="D32" s="6"/>
+      <c r="E32" s="13"/>
+      <c r="F32" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="G32" s="4"/>
-      <c r="H32" s="10"/>
+      <c r="G32" s="6"/>
+      <c r="H32" s="7"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="4" t="s">
+      <c r="A33" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="B33" s="10" t="n">
+      <c r="B33" s="7" t="n">
         <v>0.996791829147154</v>
       </c>
-      <c r="C33" s="10" t="n">
+      <c r="C33" s="7" t="n">
         <v>0.971347929011293</v>
       </c>
-      <c r="D33" s="6" t="s">
+      <c r="D33" s="8" t="s">
         <v>91</v>
       </c>
-      <c r="E33" s="13" t="n">
+      <c r="E33" s="14" t="n">
         <v>0.926779793958945</v>
       </c>
-      <c r="F33" s="4" t="s">
+      <c r="F33" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="G33" s="4"/>
-      <c r="H33" s="10"/>
+      <c r="G33" s="6"/>
+      <c r="H33" s="7"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="4" t="s">
+      <c r="A34" s="6" t="s">
         <v>93</v>
       </c>
-      <c r="B34" s="10" t="n">
+      <c r="B34" s="7" t="n">
         <v>0.974631938233094</v>
       </c>
-      <c r="C34" s="10" t="n">
+      <c r="C34" s="7" t="n">
         <v>0.987890980723224</v>
       </c>
-      <c r="D34" s="4" t="s">
+      <c r="D34" s="6" t="s">
         <v>94</v>
       </c>
-      <c r="E34" s="10" t="n">
+      <c r="E34" s="13" t="n">
         <v>0.925648389418738</v>
       </c>
-      <c r="F34" s="4" t="s">
+      <c r="F34" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="G34" s="4"/>
-      <c r="H34" s="10"/>
+      <c r="G34" s="6"/>
+      <c r="H34" s="7"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="4" t="s">
+      <c r="A35" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="B35" s="10" t="n">
+      <c r="B35" s="7" t="n">
         <v>0.987889323713514</v>
       </c>
-      <c r="C35" s="10" t="n">
+      <c r="C35" s="7" t="n">
         <v>0.977612988537665</v>
       </c>
-      <c r="D35" s="4"/>
-      <c r="E35" s="10"/>
-      <c r="F35" s="4" t="s">
+      <c r="D35" s="6"/>
+      <c r="E35" s="13"/>
+      <c r="F35" s="6" t="s">
         <v>97</v>
       </c>
-      <c r="G35" s="4"/>
-      <c r="H35" s="10"/>
+      <c r="G35" s="6"/>
+      <c r="H35" s="7"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="4" t="s">
+      <c r="A36" s="6" t="s">
         <v>98</v>
       </c>
-      <c r="B36" s="10" t="n">
+      <c r="B36" s="7" t="n">
         <v>0.999335495603225</v>
       </c>
-      <c r="C36" s="10" t="n">
+      <c r="C36" s="7" t="n">
         <v>0.992503948289454</v>
       </c>
-      <c r="D36" s="4"/>
-      <c r="E36" s="10"/>
-      <c r="F36" s="4" t="s">
+      <c r="D36" s="6"/>
+      <c r="E36" s="13"/>
+      <c r="F36" s="6" t="s">
         <v>99</v>
       </c>
-      <c r="G36" s="4" t="s">
+      <c r="G36" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="H36" s="10" t="n">
+      <c r="H36" s="7" t="n">
         <v>0.972597475309932</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="4" t="s">
+      <c r="A37" s="6" t="s">
         <v>101</v>
       </c>
-      <c r="B37" s="10" t="n">
+      <c r="B37" s="7" t="n">
         <v>0.996608992752013</v>
       </c>
-      <c r="C37" s="10" t="n">
+      <c r="C37" s="7" t="n">
         <v>0.954658409557154</v>
       </c>
-      <c r="D37" s="4"/>
-      <c r="E37" s="10"/>
-      <c r="F37" s="4" t="s">
+      <c r="D37" s="6"/>
+      <c r="E37" s="13"/>
+      <c r="F37" s="6" t="s">
         <v>102</v>
       </c>
-      <c r="G37" s="4" t="s">
+      <c r="G37" s="6" t="s">
         <v>103</v>
       </c>
-      <c r="H37" s="10" t="n">
+      <c r="H37" s="7" t="n">
         <v>0.946706660165817</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="4" t="s">
+      <c r="A38" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="B38" s="10" t="n">
+      <c r="B38" s="7" t="n">
         <v>0.953973633789916</v>
       </c>
-      <c r="C38" s="10" t="n">
+      <c r="C38" s="7" t="n">
         <v>0.820571179664792</v>
       </c>
-      <c r="D38" s="4"/>
-      <c r="E38" s="10"/>
-      <c r="F38" s="4" t="s">
+      <c r="D38" s="6"/>
+      <c r="E38" s="13"/>
+      <c r="F38" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="G38" s="4"/>
-      <c r="H38" s="10"/>
+      <c r="G38" s="6"/>
+      <c r="H38" s="7"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="4" t="s">
+      <c r="A39" s="6" t="s">
         <v>106</v>
       </c>
-      <c r="B39" s="10" t="n">
+      <c r="B39" s="7" t="n">
         <v>0.999052672382287</v>
       </c>
-      <c r="C39" s="10" t="n">
+      <c r="C39" s="7" t="n">
         <v>0.999773004244467</v>
       </c>
-      <c r="D39" s="4"/>
-      <c r="E39" s="10"/>
-      <c r="F39" s="4" t="s">
+      <c r="D39" s="6"/>
+      <c r="E39" s="13"/>
+      <c r="F39" s="6" t="s">
         <v>107</v>
       </c>
-      <c r="G39" s="4" t="s">
+      <c r="G39" s="6" t="s">
         <v>108</v>
       </c>
-      <c r="H39" s="10" t="n">
+      <c r="H39" s="7" t="n">
         <v>0.932320882916883</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="4" t="s">
+      <c r="A40" s="6" t="s">
         <v>109</v>
       </c>
-      <c r="B40" s="10" t="n">
+      <c r="B40" s="7" t="n">
         <v>0.975340833576648</v>
       </c>
-      <c r="C40" s="10" t="n">
+      <c r="C40" s="7" t="n">
         <v>0.562821812507071</v>
       </c>
-      <c r="D40" s="4"/>
-      <c r="E40" s="10"/>
-      <c r="F40" s="4" t="s">
+      <c r="D40" s="6"/>
+      <c r="E40" s="13"/>
+      <c r="F40" s="6" t="s">
         <v>110</v>
       </c>
-      <c r="G40" s="4"/>
-      <c r="H40" s="10"/>
+      <c r="G40" s="6"/>
+      <c r="H40" s="7"/>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="4" t="s">
+      <c r="A41" s="6" t="s">
         <v>111</v>
       </c>
-      <c r="B41" s="10" t="n">
+      <c r="B41" s="7" t="n">
         <v>0.996358416382452</v>
       </c>
-      <c r="C41" s="10" t="n">
+      <c r="C41" s="7" t="n">
         <v>0.857208955241132</v>
       </c>
-      <c r="D41" s="4" t="s">
+      <c r="D41" s="6" t="s">
         <v>112</v>
       </c>
-      <c r="E41" s="10" t="n">
+      <c r="E41" s="13" t="n">
         <v>0.948827781072061</v>
       </c>
-      <c r="F41" s="4" t="s">
+      <c r="F41" s="6" t="s">
         <v>113</v>
       </c>
-      <c r="G41" s="4" t="s">
+      <c r="G41" s="6" t="s">
         <v>114</v>
       </c>
-      <c r="H41" s="10" t="n">
+      <c r="H41" s="7" t="n">
         <v>0.981466622789426</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="4" t="s">
+      <c r="A42" s="6" t="s">
         <v>115</v>
       </c>
-      <c r="B42" s="10" t="n">
+      <c r="B42" s="7" t="n">
         <v>0.998096982715492</v>
       </c>
-      <c r="C42" s="10" t="n">
+      <c r="C42" s="7" t="n">
         <v>0.965794892166284</v>
       </c>
-      <c r="D42" s="4"/>
-      <c r="E42" s="10"/>
-      <c r="F42" s="4" t="s">
+      <c r="D42" s="6"/>
+      <c r="E42" s="13"/>
+      <c r="F42" s="6" t="s">
         <v>116</v>
       </c>
-      <c r="G42" s="4"/>
-      <c r="H42" s="10"/>
+      <c r="G42" s="6"/>
+      <c r="H42" s="7"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="4" t="s">
+      <c r="A43" s="6" t="s">
         <v>117</v>
       </c>
-      <c r="B43" s="10" t="n">
+      <c r="B43" s="7" t="n">
         <v>0.994235733371401</v>
       </c>
-      <c r="C43" s="10" t="n">
+      <c r="C43" s="7" t="n">
         <v>0.999915018165147</v>
       </c>
-      <c r="D43" s="4"/>
-      <c r="E43" s="10"/>
-      <c r="F43" s="4" t="s">
+      <c r="D43" s="6"/>
+      <c r="E43" s="13"/>
+      <c r="F43" s="6" t="s">
         <v>118</v>
       </c>
-      <c r="G43" s="4"/>
-      <c r="H43" s="10"/>
+      <c r="G43" s="6"/>
+      <c r="H43" s="7"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="4" t="s">
+      <c r="A44" s="6" t="s">
         <v>119</v>
       </c>
-      <c r="B44" s="10" t="n">
+      <c r="B44" s="7" t="n">
         <v>0.989972334808116</v>
       </c>
-      <c r="C44" s="10" t="n">
+      <c r="C44" s="7" t="n">
         <v>0.984044585119664</v>
       </c>
-      <c r="D44" s="4" t="s">
+      <c r="D44" s="6" t="s">
         <v>120</v>
       </c>
-      <c r="E44" s="10" t="n">
+      <c r="E44" s="13" t="n">
         <v>0.922936621639725</v>
       </c>
-      <c r="F44" s="8" t="s">
+      <c r="F44" s="10" t="s">
         <v>121</v>
       </c>
-      <c r="G44" s="8"/>
-      <c r="H44" s="12"/>
+      <c r="G44" s="10"/>
+      <c r="H44" s="11"/>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="4" t="s">
+      <c r="A45" s="6" t="s">
         <v>122</v>
       </c>
-      <c r="B45" s="10" t="n">
+      <c r="B45" s="7" t="n">
         <v>0.994871131154353</v>
       </c>
-      <c r="C45" s="10" t="n">
+      <c r="C45" s="7" t="n">
         <v>0.984978168725015</v>
       </c>
-      <c r="D45" s="4" t="s">
+      <c r="D45" s="6" t="s">
         <v>123</v>
       </c>
-      <c r="E45" s="10" t="n">
+      <c r="E45" s="13" t="n">
         <v>0.904679325010897</v>
       </c>
-      <c r="F45" s="8" t="s">
+      <c r="F45" s="10" t="s">
         <v>121</v>
       </c>
-      <c r="G45" s="8"/>
-      <c r="H45" s="12"/>
+      <c r="G45" s="10"/>
+      <c r="H45" s="11"/>
     </row>
   </sheetData>
   <mergeCells count="21">

</xml_diff>